<commit_message>
ADD: new prices from 25.09.2026
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ/ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="55">
   <si>
     <t>Дата</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Литри</t>
   </si>
   <si>
-    <t>Тип количество</t>
-  </si>
-  <si>
     <t>GTA цена</t>
   </si>
   <si>
@@ -58,151 +55,112 @@
     <t>Billing_Document</t>
   </si>
   <si>
-    <t>1147 Варна Ситроен</t>
-  </si>
-  <si>
-    <t>1911 O5 Варна</t>
-  </si>
-  <si>
-    <t>1148 Варна пристанище</t>
-  </si>
-  <si>
-    <t>1199 Varna Car Osvoboditel</t>
+    <t>Варна Цар Освободител</t>
+  </si>
+  <si>
+    <t>Варна Варненчик</t>
+  </si>
+  <si>
+    <t>Варна Евkсиноград</t>
+  </si>
+  <si>
+    <t>Варна Порт</t>
+  </si>
+  <si>
+    <t>Варна Сливница</t>
+  </si>
+  <si>
+    <t>B5383XE</t>
+  </si>
+  <si>
+    <t>B5289РХ</t>
+  </si>
+  <si>
+    <t>B4160TK</t>
+  </si>
+  <si>
+    <t>B0452TC</t>
   </si>
   <si>
     <t>B6386HH</t>
   </si>
   <si>
-    <t>B7846TP</t>
-  </si>
-  <si>
-    <t>B4160TK</t>
-  </si>
-  <si>
     <t>B8917BP</t>
   </si>
   <si>
-    <t>B0452TC</t>
-  </si>
-  <si>
-    <t>B2207PP</t>
-  </si>
-  <si>
     <t>B4161TK</t>
   </si>
   <si>
     <t>B5379XE</t>
   </si>
   <si>
-    <t>B7845TP</t>
+    <t>B9208BM</t>
+  </si>
+  <si>
+    <t>78970155027721236</t>
+  </si>
+  <si>
+    <t>78970155027721319</t>
+  </si>
+  <si>
+    <t>78970155027721293</t>
+  </si>
+  <si>
+    <t>78970155027721202</t>
   </si>
   <si>
     <t>78970155027721301</t>
   </si>
   <si>
-    <t>78970155027721194</t>
-  </si>
-  <si>
-    <t>78970155027721293</t>
-  </si>
-  <si>
     <t>78970155027721269</t>
   </si>
   <si>
-    <t>78970155027721202</t>
-  </si>
-  <si>
-    <t>78970155027721178</t>
-  </si>
-  <si>
     <t>78970155027721285</t>
   </si>
   <si>
     <t>78970155027721244</t>
   </si>
   <si>
-    <t>78970155027721251</t>
+    <t>78970155027721186</t>
   </si>
   <si>
     <t>DIESEL EKONOMY</t>
   </si>
   <si>
-    <t>95 EKONOMY UNLEADED</t>
-  </si>
-  <si>
-    <t>L15</t>
-  </si>
-  <si>
-    <t>10:29:00</t>
-  </si>
-  <si>
-    <t>13:33:00</t>
-  </si>
-  <si>
-    <t>13:31:00</t>
-  </si>
-  <si>
-    <t>13:40:00</t>
-  </si>
-  <si>
-    <t>10:13:00</t>
-  </si>
-  <si>
-    <t>13:23:00</t>
-  </si>
-  <si>
-    <t>14:11:00</t>
-  </si>
-  <si>
-    <t>13:52:00</t>
-  </si>
-  <si>
-    <t>13:29:00</t>
-  </si>
-  <si>
-    <t>13:07:00</t>
-  </si>
-  <si>
-    <t>12:33:00</t>
-  </si>
-  <si>
-    <t>10:49:00</t>
-  </si>
-  <si>
-    <t>3236508147 3236508147</t>
-  </si>
-  <si>
-    <t>3236559755 3236559755</t>
-  </si>
-  <si>
-    <t>3236606812 3236606812</t>
-  </si>
-  <si>
-    <t>3236660105 3236660105</t>
-  </si>
-  <si>
-    <t>3236661468 3236661468</t>
-  </si>
-  <si>
-    <t>3236828268 3236828268</t>
-  </si>
-  <si>
-    <t>3236878929 3236878929</t>
-  </si>
-  <si>
-    <t>3236924571 3236924571</t>
-  </si>
-  <si>
-    <t>3236924950 3236924950</t>
-  </si>
-  <si>
-    <t>3236954992 3236954992</t>
-  </si>
-  <si>
-    <t>3237075098 3237075098</t>
-  </si>
-  <si>
-    <t>3237211433 3237211433</t>
+    <t>13:35</t>
+  </si>
+  <si>
+    <t>13:38</t>
+  </si>
+  <si>
+    <t>12:47</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>10:28</t>
+  </si>
+  <si>
+    <t>10:29</t>
+  </si>
+  <si>
+    <t>13:36</t>
+  </si>
+  <si>
+    <t>12:37</t>
+  </si>
+  <si>
+    <t>14:06</t>
+  </si>
+  <si>
+    <t>11:20</t>
+  </si>
+  <si>
+    <t>13:58</t>
+  </si>
+  <si>
+    <t>13:32</t>
   </si>
   <si>
     <t>Общи литри по продукт / ДОМАШЕН СОЦИАЛЕН ПАТРОНАЖ</t>
@@ -625,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -634,17 +592,16 @@
     <col min="4" max="4" width="28.7109375" customWidth="1"/>
     <col min="5" max="5" width="22.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" customWidth="1"/>
+    <col min="11" max="11" width="7.7109375" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -684,16 +641,13 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="3">
+        <v>46266</v>
+      </c>
+      <c r="B2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="3">
-        <v>46251</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -705,36 +659,33 @@
         <v>36</v>
       </c>
       <c r="F2">
-        <v>73.44</v>
-      </c>
-      <c r="G2" t="s">
-        <v>38</v>
+        <v>40.01</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1.81</v>
       </c>
       <c r="H2" s="1">
-        <v>1.77</v>
+        <v>72.41800000000001</v>
       </c>
       <c r="I2" s="1">
-        <v>129.989</v>
+        <v>1.84</v>
       </c>
       <c r="J2" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="K2" s="1">
-        <v>132.192</v>
-      </c>
-      <c r="L2" t="s">
-        <v>39</v>
+        <v>73.61799999999999</v>
+      </c>
+      <c r="K2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>81063</v>
-      </c>
-      <c r="N2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>297703</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="3">
-        <v>46252</v>
+        <v>46266</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -749,36 +700,33 @@
         <v>36</v>
       </c>
       <c r="F3">
-        <v>56.85</v>
-      </c>
-      <c r="G3" t="s">
+        <v>61.28</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1.81</v>
+      </c>
+      <c r="H3" s="1">
+        <v>110.917</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1.84</v>
+      </c>
+      <c r="J3" s="1">
+        <v>112.755</v>
+      </c>
+      <c r="K3" t="s">
         <v>38</v>
       </c>
-      <c r="H3" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="I3" s="1">
-        <v>100.624</v>
-      </c>
-      <c r="J3" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="K3" s="1">
-        <v>102.33</v>
-      </c>
-      <c r="L3" t="s">
-        <v>40</v>
+      <c r="L3">
+        <v>322734</v>
       </c>
       <c r="M3">
-        <v>32370</v>
-      </c>
-      <c r="N3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+        <v>145672</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="3">
-        <v>46253</v>
+        <v>46267</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
@@ -793,36 +741,33 @@
         <v>36</v>
       </c>
       <c r="F4">
-        <v>42.05</v>
-      </c>
-      <c r="G4" t="s">
-        <v>38</v>
+        <v>36.74</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1.81</v>
       </c>
       <c r="H4" s="1">
-        <v>1.79</v>
+        <v>66.499</v>
       </c>
       <c r="I4" s="1">
-        <v>75.27</v>
+        <v>1.84</v>
       </c>
       <c r="J4" s="1">
-        <v>1.82</v>
-      </c>
-      <c r="K4" s="1">
-        <v>76.53100000000001</v>
-      </c>
-      <c r="L4" t="s">
-        <v>41</v>
+        <v>67.602</v>
+      </c>
+      <c r="K4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4">
+        <v>58525</v>
       </c>
       <c r="M4">
-        <v>57925</v>
-      </c>
-      <c r="N4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>148277</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="3">
-        <v>46254</v>
+        <v>46267</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -837,36 +782,33 @@
         <v>36</v>
       </c>
       <c r="F5">
-        <v>20</v>
-      </c>
-      <c r="G5" t="s">
-        <v>38</v>
+        <v>45</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1.81</v>
       </c>
       <c r="H5" s="1">
-        <v>1.81</v>
+        <v>81.45</v>
       </c>
       <c r="I5" s="1">
-        <v>36.2</v>
+        <v>1.84</v>
       </c>
       <c r="J5" s="1">
-        <v>1.84</v>
-      </c>
-      <c r="K5" s="1">
-        <v>36.8</v>
-      </c>
-      <c r="L5" t="s">
-        <v>42</v>
+        <v>82.8</v>
+      </c>
+      <c r="K5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5">
+        <v>68888</v>
       </c>
       <c r="M5">
-        <v>76960</v>
-      </c>
-      <c r="N5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+        <v>249197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="3">
-        <v>46254</v>
+        <v>46268</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
@@ -881,39 +823,36 @@
         <v>36</v>
       </c>
       <c r="F6">
-        <v>50.01</v>
-      </c>
-      <c r="G6" t="s">
-        <v>38</v>
+        <v>68.02</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1.83</v>
       </c>
       <c r="H6" s="1">
-        <v>1.81</v>
+        <v>124.477</v>
       </c>
       <c r="I6" s="1">
-        <v>90.518</v>
+        <v>1.86</v>
       </c>
       <c r="J6" s="1">
-        <v>1.84</v>
-      </c>
-      <c r="K6" s="1">
-        <v>92.018</v>
-      </c>
-      <c r="L6" t="s">
-        <v>43</v>
+        <v>126.517</v>
+      </c>
+      <c r="K6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6">
+        <v>8202</v>
       </c>
       <c r="M6">
-        <v>68230</v>
-      </c>
-      <c r="N6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>255161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="3">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
@@ -922,42 +861,39 @@
         <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F7">
-        <v>50.66</v>
-      </c>
-      <c r="G7" t="s">
-        <v>38</v>
+        <v>30</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1.83</v>
       </c>
       <c r="H7" s="1">
-        <v>1.54</v>
+        <v>54.9</v>
       </c>
       <c r="I7" s="1">
-        <v>78.01600000000001</v>
+        <v>1.86</v>
       </c>
       <c r="J7" s="1">
-        <v>1.57</v>
-      </c>
-      <c r="K7" s="1">
-        <v>79.536</v>
-      </c>
-      <c r="L7" t="s">
-        <v>44</v>
+        <v>55.8</v>
+      </c>
+      <c r="K7" t="s">
+        <v>42</v>
+      </c>
+      <c r="L7">
+        <v>77607</v>
       </c>
       <c r="M7">
-        <v>155190</v>
-      </c>
-      <c r="N7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+        <v>170066</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" s="3">
-        <v>46258</v>
+        <v>46269</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
@@ -969,215 +905,200 @@
         <v>36</v>
       </c>
       <c r="F8">
-        <v>54.27</v>
-      </c>
-      <c r="G8" t="s">
-        <v>38</v>
+        <v>55.01</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1.83</v>
       </c>
       <c r="H8" s="1">
-        <v>1.82</v>
+        <v>100.668</v>
       </c>
       <c r="I8" s="1">
-        <v>98.771</v>
+        <v>1.86</v>
       </c>
       <c r="J8" s="1">
-        <v>1.85</v>
-      </c>
-      <c r="K8" s="1">
-        <v>100.4</v>
-      </c>
-      <c r="L8" t="s">
-        <v>45</v>
+        <v>102.319</v>
+      </c>
+      <c r="K8" t="s">
+        <v>43</v>
+      </c>
+      <c r="L8">
+        <v>57117</v>
       </c>
       <c r="M8">
-        <v>56678</v>
-      </c>
-      <c r="N8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
+        <v>298617</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" s="3">
-        <v>46259</v>
+        <v>46273</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
         <v>36</v>
       </c>
       <c r="F9">
-        <v>50.02</v>
-      </c>
-      <c r="G9" t="s">
-        <v>38</v>
+        <v>24.13</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1.85</v>
       </c>
       <c r="H9" s="1">
-        <v>1.82</v>
+        <v>44.64</v>
       </c>
       <c r="I9" s="1">
-        <v>91.036</v>
+        <v>1.88</v>
       </c>
       <c r="J9" s="1">
-        <v>1.85</v>
-      </c>
-      <c r="K9" s="1">
-        <v>92.53700000000001</v>
-      </c>
-      <c r="L9" t="s">
-        <v>46</v>
+        <v>45.364</v>
+      </c>
+      <c r="K9" t="s">
+        <v>44</v>
+      </c>
+      <c r="L9">
+        <v>58726</v>
       </c>
       <c r="M9">
-        <v>8430</v>
-      </c>
-      <c r="N9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+        <v>150613</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="3">
-        <v>46259</v>
+        <v>46274</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E10" t="s">
         <v>36</v>
       </c>
       <c r="F10">
-        <v>30</v>
-      </c>
-      <c r="G10" t="s">
-        <v>38</v>
+        <v>66</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.86</v>
       </c>
       <c r="H10" s="1">
-        <v>1.82</v>
+        <v>122.76</v>
       </c>
       <c r="I10" s="1">
-        <v>54.6</v>
+        <v>1.89</v>
       </c>
       <c r="J10" s="1">
-        <v>1.85</v>
-      </c>
-      <c r="K10" s="1">
-        <v>55.5</v>
-      </c>
-      <c r="L10" t="s">
-        <v>47</v>
+        <v>124.74</v>
+      </c>
+      <c r="K10" t="s">
+        <v>45</v>
+      </c>
+      <c r="L10">
+        <v>8956</v>
       </c>
       <c r="M10">
-        <v>39497</v>
-      </c>
-      <c r="N10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+        <v>299830</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" s="3">
-        <v>46260</v>
+        <v>46279</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
         <v>36</v>
       </c>
       <c r="F11">
-        <v>38.44</v>
-      </c>
-      <c r="G11" t="s">
-        <v>38</v>
+        <v>30.02</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1.89</v>
       </c>
       <c r="H11" s="1">
-        <v>1.82</v>
+        <v>56.738</v>
       </c>
       <c r="I11" s="1">
-        <v>69.961</v>
+        <v>1.92</v>
       </c>
       <c r="J11" s="1">
-        <v>1.85</v>
-      </c>
-      <c r="K11" s="1">
-        <v>71.114</v>
-      </c>
-      <c r="L11" t="s">
-        <v>48</v>
+        <v>57.638</v>
+      </c>
+      <c r="K11" t="s">
+        <v>46</v>
+      </c>
+      <c r="L11">
+        <v>402543</v>
       </c>
       <c r="M11">
-        <v>58220</v>
-      </c>
-      <c r="N11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+        <v>150484</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" s="3">
-        <v>46262</v>
+        <v>46279</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
         <v>36</v>
       </c>
       <c r="F12">
-        <v>68</v>
-      </c>
-      <c r="G12" t="s">
-        <v>38</v>
+        <v>72.06999999999999</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1.89</v>
       </c>
       <c r="H12" s="1">
-        <v>1.82</v>
+        <v>136.212</v>
       </c>
       <c r="I12" s="1">
-        <v>123.76</v>
+        <v>1.92</v>
       </c>
       <c r="J12" s="1">
-        <v>1.85</v>
-      </c>
-      <c r="K12" s="1">
-        <v>125.8</v>
-      </c>
-      <c r="L12" t="s">
-        <v>49</v>
+        <v>138.374</v>
+      </c>
+      <c r="K12" t="s">
+        <v>47</v>
+      </c>
+      <c r="L12">
+        <v>82666</v>
       </c>
       <c r="M12">
-        <v>77403</v>
-      </c>
-      <c r="N12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+        <v>150565</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" s="3">
-        <v>46265</v>
+        <v>46280</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
         <v>18</v>
@@ -1191,34 +1112,31 @@
       <c r="F13">
         <v>40</v>
       </c>
-      <c r="G13" t="s">
-        <v>38</v>
+      <c r="G13" s="1">
+        <v>1.89</v>
       </c>
       <c r="H13" s="1">
-        <v>1.81</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="I13" s="1">
-        <v>72.40000000000001</v>
+        <v>1.92</v>
       </c>
       <c r="J13" s="1">
-        <v>1.84</v>
-      </c>
-      <c r="K13" s="1">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="L13" t="s">
-        <v>50</v>
+        <v>76.8</v>
+      </c>
+      <c r="K13" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13">
+        <v>5390</v>
       </c>
       <c r="M13">
-        <v>81700</v>
-      </c>
-      <c r="N13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
+        <v>150924</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" s="4" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1228,22 +1146,22 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="5" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1251,57 +1169,37 @@
         <v>36</v>
       </c>
       <c r="B18" s="7">
-        <v>523.08</v>
+        <v>568.28</v>
       </c>
       <c r="C18" s="8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D18" s="9">
-        <v>1.80303</v>
+        <v>1.84289</v>
       </c>
       <c r="E18" s="7">
-        <v>943.13</v>
+        <v>1047.28</v>
       </c>
       <c r="F18" s="7">
-        <v>958.8200000000001</v>
+        <v>1064.33</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19" s="7">
-        <v>50.66</v>
-      </c>
-      <c r="C19" s="8">
-        <v>1</v>
-      </c>
-      <c r="D19" s="9">
-        <v>1.53999</v>
-      </c>
-      <c r="E19" s="7">
-        <v>78.02</v>
-      </c>
-      <c r="F19" s="7">
-        <v>79.54000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="B20" s="11">
-        <v>573.74</v>
-      </c>
-      <c r="C20" s="12">
+      <c r="A19" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="11">
+        <v>568.28</v>
+      </c>
+      <c r="C19" s="12">
         <v>12</v>
       </c>
-      <c r="D20" s="9"/>
-      <c r="E20" s="11">
-        <v>1021.15</v>
-      </c>
-      <c r="F20" s="11">
-        <v>1038.36</v>
+      <c r="D19" s="9"/>
+      <c r="E19" s="11">
+        <v>1047.28</v>
+      </c>
+      <c r="F19" s="11">
+        <v>1064.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>